<commit_message>
sim: the Sage holds her spells, keeps two buffs up and attacks
The model gave her no attack and five buffs to keep up, so she dealt none of the damage of the party and won less than an attacker in her place. With the spells of the Magic User she was, Circle Protect and Circle Brave and then her spells, she wins as an attacker does. The measures that hold a Sage are regenerated.
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -18242,7 +18242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19686,7 +19686,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -19700,7 +19700,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 138: the Sage raises the abilities of the party (Circle Brave kept up) | last since 2026-10-11: the attack buff serves the fewest members of the parties a Sage is in</t>
+          <t>atwiki dt2-2 page 138: the Sage raises the abilities of the party (Circle Brave kept up) | last since 2026-10-11: the attack buff serves the fewest members of the parties a Sage is in | 2026-10-13 : second, after Circle Protect: at the end of the list she never came to cast it. Sun Veil, Amplify and Accelerator left her rules the same day: each added nothing that could be measured at C30, C36, C38, C40 and P24 (150 battles, with and without each), and with the five kept up she never attacked. With the two buffs and then her spells she wins 90% of those fights in the last place of the reference party, against 87%</t>
         </is>
       </c>
     </row>
@@ -19736,7 +19736,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -19745,23 +19745,23 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>status:163</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Sun Veil kept up</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>sage</t>
+          <t>shooter</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -19770,48 +19770,48 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>status:172</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Amplify kept up</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>sage</t>
+          <t>soul summoner</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>doll_slot_free</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>status:168</t>
+          <t>doll:Mercidarian|Spartan|Musiy|Catalina|Oracles</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Accelerator (one ally, 3 turns) after the party-wide buffs</t>
+          <t>atwiki dt2-2 pages 131, 146: both doll slots kept filled; GameFAQs Class Skill info - Spieler: Mercidarian by far the best doll</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>sage</t>
+          <t>soul summoner</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -19832,7 +19832,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>shooter</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -19840,67 +19840,67 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>soul summoner</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>doll_slot_free</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>doll:Mercidarian|Spartan|Musiy|Catalina|Oracles</t>
+          <t>status:170</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 pages 131, 146: both doll slots kept filled; GameFAQs Class Skill info - Spieler: Mercidarian by far the best doll</t>
+          <t>atwiki dt2-2 page 133: the Valkyrie draws attacks as the wall of the party</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>soul summoner</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>party_hp_below:0.5</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>atwiki dt2-2 page 133</t>
         </is>
       </c>
     </row>
@@ -19911,21 +19911,21 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>status:162</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>atwiki dt2-2 page 122: the Paladin uses herself as the shield of the party (Protect kept up on the weakest member)</t>
         </is>
       </c>
     </row>
@@ -19936,7 +19936,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -19945,87 +19945,87 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>status:170</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 133: the Valkyrie draws attacks as the wall of the party</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>treasure hunter</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>party_hp_below:0.5</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 133</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "can help with items in emergency situations"</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>treasure hunter</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>status:162</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 122: the Paladin uses herself as the shield of the party (Protect kept up on the weakest member)</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>treasure hunter</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_hp_below:0.35</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>heal:0.35</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>GameFAQs faqs/80834, Recommended Party: items in an emergency</t>
         </is>
       </c>
     </row>
@@ -20036,96 +20036,96 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "can help with items in emergency situations"</t>
+          <t>GameFAQs faqs/80834, Recommended Party: Pursuit Stab as the core</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>treasure hunter</t>
+          <t>valkyrie</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>treasure hunter</t>
+          <t>valkyrie</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ally_hp_below:0.35</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>heal:0.35</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: items in an emergency</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>treasure hunter</t>
+          <t>valkyrie</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>party_hp_below:0.5</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: Pursuit Stab as the core</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "in serious bosses she should usually be supporting"</t>
         </is>
       </c>
     </row>
@@ -20136,21 +20136,21 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>status:183</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the guard buffs of the party</t>
         </is>
       </c>
     </row>
@@ -20161,21 +20161,21 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>status:161</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>GameFAQs faqs/80834, Recommended Party: War Cry maxed early</t>
         </is>
       </c>
     </row>
@@ -20186,21 +20186,21 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>party_hp_below:0.5</t>
+          <t>boss</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>status:180</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "in serious bosses she should usually be supporting"</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the Valkyrie prebuffs Parry and Cover in hard fights</t>
         </is>
       </c>
     </row>
@@ -20211,21 +20211,21 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>boss</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>status:183</t>
+          <t>status:171</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the guard buffs of the party</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the Valkyrie prebuffs Parry and Cover in hard fights</t>
         </is>
       </c>
     </row>
@@ -20236,7 +20236,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -20245,98 +20245,98 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>status:161</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: War Cry maxed early</t>
+          <t>GameFAQs faqs/80834, Recommended Party: Daedalus, "one of the best fire and forget nukes"</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>mage</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>6</v>
+        <v>0.5</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>boss</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>status:180</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the Valkyrie prebuffs Parry and Cover in hard fights</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>sage</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>boss</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>status:171</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the Valkyrie prebuffs Parry and Cover in hard fights</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>healer</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: Daedalus, "one of the best fire and forget nukes"</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>mage</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -20357,11 +20357,11 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>sage</t>
+          <t>magical princess</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>2.5</v>
+        <v>0.5</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -20382,11 +20382,11 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>healer</t>
+          <t>mistress</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -20407,11 +20407,11 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>soul summoner</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -20432,7 +20432,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>magical princess</t>
+          <t>dolls</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -20457,7 +20457,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>mistress</t>
+          <t>attacker</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -20482,7 +20482,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>soul summoner</t>
+          <t>kunoichi</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -20507,7 +20507,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>dolls</t>
+          <t>shooter</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -20532,7 +20532,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>attacker</t>
+          <t>joker</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -20549,81 +20549,6 @@
         </is>
       </c>
       <c r="E92" t="inlineStr">
-        <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>kunoichi</t>
-        </is>
-      </c>
-      <c r="B93" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>ally_tp_below:0.15</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>tp:0.15</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>shooter</t>
-        </is>
-      </c>
-      <c r="B94" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>ally_tp_below:0.15</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>tp:0.15</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>joker</t>
-        </is>
-      </c>
-      <c r="B95" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>ally_tp_below:0.15</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>tp:0.15</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
         <is>
           <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
         </is>
@@ -21687,7 +21612,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Heal; Circle Brave; Circle Protect; Accelerator; Amplify; Sun Veil; Dispel; Esarhaddon; Slow; Stab Guard; Slash Guard; Bash Guard; Prism Dawn; Fast Cast; Sleep; Silence</t>
+          <t>Heal; Circle Brave; Circle Protect; Fireball; Ice Edge; Thunderbolt; Air Cutter; Stone Hammer; Accelerator; Amplify; Sun Veil; Dispel; Esarhaddon; Slow; Stab Guard; Slash Guard; Bash Guard; Prism Dawn; Fast Cast; Sleep; Silence; Bible Thump</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -21697,7 +21622,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 138 (support: party buffs, ailments, automatic cure); GameFAQs faqs/80834 (Hentaicheg), Class Skill info pages</t>
+          <t>atwiki dt2-2 page 138 (support: party buffs, ailments, automatic cure); GameFAQs faqs/80834 (Hentaicheg), Class Skill info pages | 2026-10-13 : she holds the five spells of the Magic User she was and Bible Thump (the classes of her path learn them); without them she dealt none of the damage of the party</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sim: three habits of a player for the members who heal
A member whose rules heal keeps the TP of two heals back from her buffs and attacks; a buff of the whole party is cast again when half of its members lack it; and she defends in the place of striking with a plain blow an enemy that answers it (Avenger, Dark Aura). Without them the healer and the Sage of the party Mage-Heavy, out of TP, hit the last boss with their staffs and were struck back: 45% of wins with the faster chant of the Sage, 82% with the habits.
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -17290,7 +17290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -18228,6 +18228,46 @@
       <c r="D46" t="inlineStr">
         <is>
           <t>docs/generated/GUIDE_CURVE.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>heal_reserve_casts</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>TP a member whose rules heal keeps back from her buffs and attacks: this many casts of her cheapest heal (sim/policy.py heal_reserve)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>choice (2026-10-13): what a player who is the heal of a party does; without it the Sage of the party Mage-Heavy spent the TP of the party on Fireball and on casting her buffs again</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>party_buff_recast_share</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>A buff of the whole party is cast again when at least this share of its members lack it</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>choice (2026-10-13): one member who lost it alone does not call for 22 TP</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sim: no member strikes a punished blow that is worth nothing
A plain blow on an enemy with Avenger or Dark Aura that would take less than a hundredth of its HP is not struck: the member defends. The members of the party Anti-Meta-Plus, out of TP at C30, hit a boss with Dark Aura fifty times a fight for none of the damage and lost a tenth of every stat each time: 70% of wins, 96% with the habit.
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -17290,7 +17290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -18268,6 +18268,26 @@
       <c r="D48" t="inlineStr">
         <is>
           <t>choice (2026-10-13): one member who lost it alone does not call for 22 TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>punished_blow_floor</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>A plain blow that takes less than this share of the max HP of an enemy with Avenger or Dark Aura is not struck: the member defends (sim/policy.py weak_blow)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>choice (2026-10-13): a blow worth less than a hundredth of the boss is not worth a tenth of every stat</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: readings of Cleanse and Heaven or Hell Effect in the audit
Both act in the simulator; the prepared battle of the audit cannot show
them (the cure is aimed at a member with no ailment, the heal at foes at
full HP). Aimed where they can act, Cleanse removes poison and sleep and
Heaven or Hell Effect heals 10% of max HP under its cap. Checklist 117
of 130.

etoile_dances.py also measures Debilitating Salsa in pairs.
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -9892,7 +9892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11558,6 +11558,40 @@
       <c r="C98" t="inlineStr">
         <is>
           <t>The party of the sheets wins 0% at level 99 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. Even with a crown bonus of 50 it wins 0%: the fight asks for an answer the policy does not play (sheet PostgameBosses, what the pages say). Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>34 Cleanse</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>A cure aimed at one ally: the prepared battle aims it at a member with no ailment. Aimed at the member poisoned and asleep it removes both (probe_two_actives_2026-10-15.py, recheck 2026-10-15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>142 Heaven or Hell Effect</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>The heal of a random move, aimed at a foe: the prepared foes are at full HP. A foe at half HP regains 10% of its max HP, under the cap of 555 (probe_two_actives_2026-10-15.py, recheck 2026-10-15).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sim: the Etoile keeps Waltz and Salsa up instead of Waltz and Mazurka
Measured with measures/etoile_dances.py at C22 - C40 and P24, 200
battles a pair: the same wins, fights 5 - 33% shorter. It is how the
model plays her, in the game and in the variant alike; no value of the
mod changes.

Full suite again: curve 34 of 44, battery 79 of 85, classes 74 of 76,
unchanged. The Juggernaut party, which holds her, wins more in both
(game 48% > 57%, variant 67% > 72%). Audit readings of her dances
follow the new pair; checklist 117 of 130.
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -10673,14 +10673,14 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Her two dance slots hold Fascinating Waltz and Dumbing Mazurka (rules status:195, 201).</t>
+          <t>Her two dance slots hold Fascinating Waltz and Debilitating Salsa (rules status:195, 199).</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>usage etoile | Debilitating Salsa</t>
+          <t>usage etoile | Dumbing Mazurka</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -10690,7 +10690,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Her two dance slots hold Fascinating Waltz and Dumbing Mazurka.</t>
+          <t>Her two dance slots hold Fascinating Waltz and Debilitating Salsa (rules status:195, 199). Waltz and Salsa win as often as Waltz and Mazurka and end the fights 5 - 33% sooner at C22 - C40 and P24 (measures/etoile_dances.py, 2026-10-15).</t>
         </is>
       </c>
     </row>
@@ -10707,7 +10707,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Her two dance slots hold Fascinating Waltz and Dumbing Mazurka.</t>
+          <t>Her two dance slots hold Fascinating Waltz and Debilitating Salsa (rules status:195, 199).</t>
         </is>
       </c>
     </row>
@@ -10724,7 +10724,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Her two dance slots hold Fascinating Waltz and Dumbing Mazurka.</t>
+          <t>Her two dance slots hold Fascinating Waltz and Debilitating Salsa (rules status:195, 199).</t>
         </is>
       </c>
     </row>
@@ -10741,7 +10741,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Her two dance slots hold Fascinating Waltz and Dumbing Mazurka.</t>
+          <t>Her two dance slots hold Fascinating Waltz and Debilitating Salsa (rules status:195, 199).</t>
         </is>
       </c>
     </row>
@@ -18889,12 +18889,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>status:201</t>
+          <t>status:199</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Dumbing Mazurka on the enemies</t>
+          <t>Debilitating Salsa on the enemies</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: the last readings of the audit; checklist 130 of 130
Absolute Attack and Barrage find nothing to act on at C38; Spartan
comes after Mercidarian in the doll order; Accelerator, Amplify and
Sun Veil left the rules of the Sage on 2026-10-13; Bible Thump and
Phoenix need a weapon the role does not hold. Also the scripts of two
measures of 2026-10-16: the Juggernaut party and C36 with more ATK.
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -9892,7 +9892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11592,6 +11592,142 @@
       <c r="C100" t="inlineStr">
         <is>
           <t>The heal of a random move, aimed at a foe: the prepared foes are at full HP. A foe at half HP regains 10% of its max HP, under the cap of 555 (probe_two_actives_2026-10-15.py, recheck 2026-10-15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>276 Absolute Attack</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Effect 307 cancels the answers of the target to a blow (Avenger 249, Counter Whip 303, effect 250, the unique skill 447). Samael (C38) has none of them, so nothing changes there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>302 Barrage</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Effect 251 adds two hits to a plain attack only. At C38 the skills of the Kunoichi always score above her plain attack, so she never makes one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>usage soul summoner | Spartan</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>doll order</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Her rule fills both doll slots in the order Mercidarian, Spartan, Musiy, Catalina, Oracles: Mercidarian takes both slots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>usage sage | Accelerator</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>role choice</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Left out of her rules on 2026-10-13 (sheet Policies, rule status:161): each added nothing that could be measured at C30, C36, C38, C40 and P24 (150 battles, with and without each), and with all five kept up she never attacked. She keeps Circle Protect and Circle Brave, then casts her spells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>usage sage | Amplify</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>role choice</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Left out of her rules on 2026-10-13 (sheet Policies, rule status:161): each added nothing that could be measured at C30, C36, C38, C40 and P24 (150 battles, with and without each), and with all five kept up she never attacked. She keeps Circle Protect and Circle Brave, then casts her spells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>usage sage | Sun Veil</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>role choice</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Left out of her rules on 2026-10-13 (sheet Policies, rule status:161): each added nothing that could be measured at C30, C36, C38, C40 and P24 (150 battles, with and without each), and with all five kept up she never attacked. She keeps Circle Protect and Circle Brave, then casts her spells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>usage sage | Bible Thump</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>role choice</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>A tome skill: the Sage of the model holds no tome.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>usage kunoichi | Phoenix</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>role choice</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>A projectile skill: the Kunoichi of the model holds a Tantou.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: the Python simulator removed; the C# engine is the only one
The engine was proven equal to sim/ trace by trace and now stands alone:
- the data readers (data, setup, variant, progression) moved to
  gamedata/, with the reference levels of the checkpoints (levels.py);
- removed: sim/, engine_cs/parity, the Python measure tools of tools/
  and measures/ (their reports are written by dtcli suite), the bridge
  engine_client.py and the tests of the simulator;
- the calibration rows K01 - K05 and K08 are C# tests
  (CalibrationTests.cs), K06 - K08 data tests in test_calibration.py;
  the golden files of the engine tests are kept with them;
- sim_coverage.py reads the engine's coverage from
  data_tables/engine_coverage.json and finds the C# tests;
- tools/engine_golden.py checks a change of the engine against its own
  recorded traces with no Python tool.
Full suite: 8 of 8 steps, every report as before; dotnet test 14 of 14.
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -9581,7 +9581,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>test_sim_formulas.TurnOrder</t>
+          <t>engine_cs CalibrationTests.K01_TurnOrderReproducesTheSpeedTestOfTheJapaneseWiki</t>
         </is>
       </c>
     </row>
@@ -9618,7 +9618,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>test_sim_calibration.ChantSpeed</t>
+          <t>engine_cs CalibrationTests.K02_EachPieceShortensTheChantUntilTheThird</t>
         </is>
       </c>
     </row>
@@ -9655,7 +9655,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>test_sim_calibration.CriticalFactor</t>
+          <t>engine_cs CalibrationTests.K03_TheSealbookTestFitsAQuarterMore</t>
         </is>
       </c>
     </row>
@@ -9692,7 +9692,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>test_sim_calibration.DaedalusAttack</t>
+          <t>engine_cs CalibrationTests.K04_EveryMeasuredDaedalusAttackFallsInTheRangeOfTheFormula</t>
         </is>
       </c>
     </row>
@@ -9729,7 +9729,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>test_sim_calibration.SummonStats</t>
+          <t>engine_cs CalibrationTests.K05_SummonStatsAreTheBestOfThePartyTimesTheFactorOfTheForm</t>
         </is>
       </c>
     </row>
@@ -9766,7 +9766,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>test_sim_calibration.ChantStat</t>
+          <t>test_calibration.ChantStat</t>
         </is>
       </c>
     </row>
@@ -9803,7 +9803,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>test_sim_calibration.EncounterSteps</t>
+          <t>test_calibration.EncounterSteps</t>
         </is>
       </c>
     </row>
@@ -9840,7 +9840,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>test_sim_calibration.GenerousHeart</t>
+          <t>test_calibration.GenerousHeart; engine_cs CalibrationTests.K08_MaidMasteryTakesGenerousHeartTo22Percent</t>
         </is>
       </c>
     </row>
@@ -9877,7 +9877,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>tools/sim_anchors.py N05, N06</t>
+          <t>dtcli sim-anchors N05, N06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sim[policy]: the Dark Lord keeps Berserk up before Power Charge
With the charge first, the charged turn went to Berserk and the charge was lost (dtcli trace C29). Power Charge adds 1.05 - 1.3 to the other bonus of the next physical blow (x2.05 - x2.3). Both sides: curve 35 of 44 within (was 33), battery 79 of 85 (was 78).
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -18691,7 +18691,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -18705,7 +18705,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "the rotation is Power Charge &gt; Nuke"</t>
+          <t>Berserk kept up before Power Charge, so that the turn after the charge is a blow (2026-10-16: with the charge first, the charged turn went to Berserk; dtcli trace C29 Meta)</t>
         </is>
       </c>
     </row>
@@ -18716,7 +18716,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
sim[roles]: the maid role plays as the diva; suite: unique-battery, charts
The maid role, whose path ends in the Diva, takes the skill plan and the Leather Shield of the diva role and plays by its policy rows (heal at 35%, the heal and speed songs, TP after them); a row or a plan entry the classes so far cannot use is skipped, so she is still a Maid at the start. With her own rows the Diva of that role won 28% at C40 in class-stages, now 70% (diva role 71%); class-stages 68 of 76 rows within; party battery 79 of 85.

The suite runs unique-battery, and tools/class_charts.py draws docs/generated/charts/class_balance.png and class_stages.png from the reports (by stage: attackers by length, supports and tanks by wins, or by length where every fight is won).
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -18472,7 +18472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E92"/>
+  <dimension ref="A1:E93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19530,7 +19530,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>GameFAQs faqs/80834, Recommended Party: items when a member falls | 2026-10-16: the maid role plays by the rows of the diva role (her path ends in the Diva; class-stages C40 28% with her own rows)</t>
         </is>
       </c>
     </row>
@@ -19545,17 +19545,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ally_hp_below:0.5</t>
+          <t>ally_hp_below:0.35</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>heal:0.35</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 120: the Maid restores HP and TP at no cost</t>
+          <t>GameFAQs faqs/80834, Recommended Party: First Aid or an item in an emergency | 2026-10-16: the maid role plays by the rows of the diva role (her path ends in the Diva; class-stages C40 28% with her own rows)</t>
         </is>
       </c>
     </row>
@@ -19570,17 +19570,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.4</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>tp:0.4</t>
+          <t>status:215</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 120</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "upkeeps Heal/Speed song in boss battles"; the heal song first | 2026-10-16: the maid role plays by the rows of the diva role (her path ends in the Diva; class-stages C40 28% with her own rows)</t>
         </is>
       </c>
     </row>
@@ -19600,12 +19600,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>status:215</t>
+          <t>status:217</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 129: Replenishing Carol</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the speed song | 2026-10-16: the maid role plays by the rows of the diva role (her path ends in the Diva; class-stages C40 28% with her own rows)</t>
         </is>
       </c>
     </row>
@@ -19620,42 +19620,42 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_tp_below:0.35</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>tp:0.35</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "helps manage the party TP with cook and self sacrifice" | 2026-10-16: the maid role plays by the rows of the diva role (her path ends in the Diva; class-stages C40 28% with her own rows)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>mistress</t>
+          <t>maid</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Resurrect or items</t>
+          <t>the mean damage per time of every skill | 2026-10-16: the maid role plays by the rows of the diva role (her path ends in the Diva; class-stages C40 28% with her own rows)</t>
         </is>
       </c>
     </row>
@@ -19666,21 +19666,21 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>status:215</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>the heal song kept up</t>
+          <t>Resurrect or items</t>
         </is>
       </c>
     </row>
@@ -19691,7 +19691,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -19700,12 +19700,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>status:161</t>
+          <t>status:215</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>War Cry kept up</t>
+          <t>the heal song kept up</t>
         </is>
       </c>
     </row>
@@ -19716,7 +19716,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -19725,37 +19725,37 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:161</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>War Cry kept up</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>papillon</t>
+          <t>mistress</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -19766,21 +19766,21 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
@@ -19791,46 +19791,46 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the best area attack and the damage of the party</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>sage</t>
+          <t>papillon</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the best area attack and the damage of the party</t>
         </is>
       </c>
     </row>
@@ -19841,21 +19841,21 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>party_hp_below:0.5</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>heals when the party is low</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
@@ -19866,21 +19866,21 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>enemy_buffed</t>
+          <t>party_hp_below:0.5</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>dispel</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Dispel against boss buffs</t>
+          <t>heals when the party is low</t>
         </is>
       </c>
     </row>
@@ -19891,21 +19891,21 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>boss</t>
+          <t>enemy_buffed</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ailment:122;117;116</t>
+          <t>dispel</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 138: the Sage supports with ailment spells; slow, silence and sleep in that order (page 227 names slow and silence against the heal wall of Calliope)</t>
+          <t>Dispel against boss buffs</t>
         </is>
       </c>
     </row>
@@ -19916,21 +19916,21 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>boss</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>status:161</t>
+          <t>ailment:122;117;116</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 138: the Sage raises the abilities of the party (Circle Brave kept up) | last since 2026-10-11: the attack buff serves the fewest members of the parties a Sage is in | 2026-10-13 : second, after Circle Protect: at the end of the list she never came to cast it. Sun Veil, Amplify and Accelerator left her rules the same day: each added nothing that could be measured at C30, C36, C38, C40 and P24 (150 battles, with and without each), and with the five kept up she never attacked. With the two buffs and then her spells she wins 90% of those fights in the last place of the reference party, against 87%</t>
+          <t>atwiki dt2-2 page 138: the Sage supports with ailment spells; slow, silence and sleep in that order (page 227 names slow and silence against the heal wall of Calliope)</t>
         </is>
       </c>
     </row>
@@ -19941,7 +19941,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -19950,12 +19950,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>status:162</t>
+          <t>status:161</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 138 (Circle Protect kept up)</t>
+          <t>atwiki dt2-2 page 138: the Sage raises the abilities of the party (Circle Brave kept up) | last since 2026-10-11: the attack buff serves the fewest members of the parties a Sage is in | 2026-10-13 : second, after Circle Protect: at the end of the list she never came to cast it. Sun Veil, Amplify and Accelerator left her rules the same day: each added nothing that could be measured at C30, C36, C38, C40 and P24 (150 battles, with and without each), and with the five kept up she never attacked. With the two buffs and then her spells she wins 90% of those fights in the last place of the reference party, against 87%</t>
         </is>
       </c>
     </row>
@@ -19966,7 +19966,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -19975,23 +19975,23 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:162</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>atwiki dt2-2 page 138 (Circle Protect kept up)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>shooter</t>
+          <t>sage</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -20012,7 +20012,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>soul summoner</t>
+          <t>shooter</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -20020,17 +20020,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>doll_slot_free</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>doll:Mercidarian|Spartan|Musiy|Catalina|Oracles</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 pages 131, 146: both doll slots kept filled; GameFAQs Class Skill info - Spieler: Mercidarian by far the best doll</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -20041,46 +20041,46 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>doll_slot_free</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>doll:Mercidarian|Spartan|Musiy|Catalina|Oracles</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>atwiki dt2-2 pages 131, 146: both doll slots kept filled; GameFAQs Class Skill info - Spieler: Mercidarian by far the best doll</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>soul summoner</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -20091,21 +20091,21 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>status:170</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 133: the Valkyrie draws attacks as the wall of the party</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
@@ -20116,21 +20116,21 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>party_hp_below:0.5</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>status:170</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 133</t>
+          <t>atwiki dt2-2 page 133: the Valkyrie draws attacks as the wall of the party</t>
         </is>
       </c>
     </row>
@@ -20141,21 +20141,21 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>party_hp_below:0.5</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>status:162</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 122: the Paladin uses herself as the shield of the party (Protect kept up on the weakest member)</t>
+          <t>atwiki dt2-2 page 133</t>
         </is>
       </c>
     </row>
@@ -20166,7 +20166,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -20175,37 +20175,37 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:162</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>atwiki dt2-2 page 122: the Paladin uses herself as the shield of the party (Protect kept up on the weakest member)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>treasure hunter</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "can help with items in emergency situations"</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -20216,21 +20216,21 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "can help with items in emergency situations"</t>
         </is>
       </c>
     </row>
@@ -20241,21 +20241,21 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ally_hp_below:0.35</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>heal:0.35</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: items in an emergency</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
@@ -20266,46 +20266,46 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_hp_below:0.35</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>heal:0.35</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: Pursuit Stab as the core</t>
+          <t>GameFAQs faqs/80834, Recommended Party: items in an emergency</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>treasure hunter</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>GameFAQs faqs/80834, Recommended Party: Pursuit Stab as the core</t>
         </is>
       </c>
     </row>
@@ -20316,21 +20316,21 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
@@ -20341,21 +20341,21 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>party_hp_below:0.5</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "in serious bosses she should usually be supporting"</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
@@ -20366,21 +20366,21 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>party_hp_below:0.5</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>status:183</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the guard buffs of the party</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "in serious bosses she should usually be supporting"</t>
         </is>
       </c>
     </row>
@@ -20391,7 +20391,7 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -20400,12 +20400,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>status:161</t>
+          <t>status:183</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: War Cry maxed early</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the guard buffs of the party</t>
         </is>
       </c>
     </row>
@@ -20416,21 +20416,21 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>boss</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>status:180</t>
+          <t>status:161</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the Valkyrie prebuffs Parry and Cover in hard fights</t>
+          <t>GameFAQs faqs/80834, Recommended Party: War Cry maxed early</t>
         </is>
       </c>
     </row>
@@ -20441,7 +20441,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -20450,7 +20450,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>status:171</t>
+          <t>status:180</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -20466,57 +20466,57 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>boss</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:171</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: Daedalus, "one of the best fire and forget nukes"</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the Valkyrie prebuffs Parry and Cover in hard fights</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>mage</t>
+          <t>valkyrie</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>0.5</v>
+        <v>8</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
+          <t>GameFAQs faqs/80834, Recommended Party: Daedalus, "one of the best fire and forget nukes"</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>sage</t>
+          <t>mage</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>2.5</v>
+        <v>0.5</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -20537,7 +20537,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>healer</t>
+          <t>sage</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -20562,11 +20562,11 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>healer</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -20587,11 +20587,11 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>magical princess</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -20612,11 +20612,11 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>mistress</t>
+          <t>magical princess</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -20637,11 +20637,11 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>soul summoner</t>
+          <t>mistress</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -20662,7 +20662,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>dolls</t>
+          <t>soul summoner</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -20687,11 +20687,11 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>attacker</t>
+          <t>dolls</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -20712,11 +20712,11 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>kunoichi</t>
+          <t>attacker</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -20737,7 +20737,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>shooter</t>
+          <t>kunoichi</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -20762,23 +20762,48 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
+          <t>shooter</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.15</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>tp:0.15</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
           <t>joker</t>
         </is>
       </c>
-      <c r="B92" t="n">
+      <c r="B93" t="n">
         <v>1.5</v>
       </c>
-      <c r="C92" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>ally_tp_below:0.15</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr">
+      <c r="D93" t="inlineStr">
         <is>
           <t>tp:0.15</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr">
+      <c r="E93" t="inlineStr">
         <is>
           <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
         </is>
@@ -21041,7 +21066,11 @@
           <t>Megaphone</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Leather Shield</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Leather Helmet</t>
@@ -21074,7 +21103,12 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 pages 120, 129, 143</t>
+          <t>atwiki dt2-2 pages 120, 129, 143 | 2026-10-16: the skill plan and the Leather Shield of the diva role (GameFAQs faqs/80834, Hentaicheg), with the Maid skills of the start kept: with the priority list alone the Diva of this role won 28% at C40 (class-stages) against 71%.</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Replenishing Carol:max; Self Session:1; Song Mastery:max; First Aid:3; Cook:3; Generous Heart:3; Maid Mastery:3; Lightning March:3; Blissful Chorale:3; Maid Mastery:max; Generous Heart:max; Cook:max; First Aid:max; Lightning March:max; Concentration Prelude:max; Auto-Recovery:max; Fast Talk:max</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: no file names the removed Python simulator as current
Comments, docstrings and workbook notes point at the engine (engine_cs) or gamedata/ where they named sim/.
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -472,7 +472,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Every choice of the simulator of phase 1 (sim/) that is not a figure of the game: the policies of the party, the reference parties and their builds, the checkpoints, the settings of a run, the calibration tests and the assumptions the model still rests on. Figures of the game are read by sim/data.py from the game files; constants of the program stay in sim/formulas.py with their address.</t>
+          <t>Every choice of the battle model that is not a figure of the game: the policies of the party, the reference parties and their builds, the checkpoints, the settings of a run, the calibration tests and the assumptions the model still rests on. Figures of the game are read by gamedata/data.py from the game files; constants of the program stay in engine_cs/src/DtEngine/Formulas.cs with their address.</t>
         </is>
       </c>
     </row>
@@ -18826,7 +18826,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Battles played for each checkpoint a change touches, in vanilla and with the change (sim/measures.py check_change)</t>
+          <t>Battles played for each checkpoint a change touches, in vanilla and with the change (Measures.cs CheckChange)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -18966,7 +18966,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Most random battles in a row an expedition measure plays (sim/measures.py expedition)</t>
+          <t>Most random battles in a row an expedition measure plays (Measures.cs Expedition)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -19106,7 +19106,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>a role casts an ailment on an enemy only when its roll has at least this chance against the enemy's resistance (sim/policy.py act_ailment)</t>
+          <t>a role casts an ailment on an enemy only when its roll has at least this chance against the enemy's resistance (Policy.cs)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -19456,7 +19456,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>TP a member whose rules heal keeps back from her buffs and attacks: this many casts of her cheapest heal (sim/policy.py heal_reserve)</t>
+          <t>TP a member whose rules heal keeps back from her buffs and attacks: this many casts of her cheapest heal (Policy.cs)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -19496,7 +19496,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>A plain blow that takes less than this share of the max HP of an enemy with Avenger or Dark Aura is not struck: the member defends (sim/policy.py weak_blow)</t>
+          <t>A plain blow that takes less than this share of the max HP of an enemy with Avenger or Dark Aura is not struck: the member defends (Policy.cs)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">

</xml_diff>

<commit_message>
balance: six bosses back toward the game's difficulty
dtcli boss-fit on the corrected engine, gentle pairs that keep every
archetype of the battery inside its share: C14 HP x1.2 with ATK and
INT x1.08, C15 HP x1.3, C29 HP x1.3 (now played with the guide's
preparation, so taken off the skip list), C35 HP x1.2, C37 HP x1.1
with ATK and INT x1.08, C39 HP x1.1. Curve 39 of 44 within the
windows of the game (34 before), 5 easier and 0 harder; the five
left alone have their reason in BOSS_FIT.md (an archetype under its
floor in the game already, or any pair breaking one).
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -19478,14 +19478,10 @@
           <t>boss_fit_skip</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>C29</t>
-        </is>
-      </c>
+      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Checkpoints tools/boss_fit.py gentle leaves alone: the model does not play them as the guide describes (docs/generated/GUIDE_CURVE.md, "read: policy gap")</t>
+          <t>Checkpoints tools/boss_fit.py gentle leaves alone: none since 2026-10-19 (C29 is played with the guide's preparation, sheet CheckpointGuests)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">

</xml_diff>

<commit_message>
data: readings of the six postgame bosses the corrected engine moved
P05, P25, P28, P31, P44, P52: a preparation gap; with a crown bonus of 40 (the stand-in for a player's preparation) the party wins 87 - 100% (dtcli crown-trial). Guide curve: 0 below and unread.
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -9894,7 +9894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11747,6 +11747,108 @@
       <c r="C109" t="inlineStr">
         <is>
           <t>At C18 the songs of the maid role (a Bard, level 29) already keep the party at full HP and TP, so a larger song bonus changes no fight there. It serves where HP or TP run short: the skill battery reads it niche (best cell C38 boss, Mage-Heavy, fights 16% shorter; 2026-10-17). Unread since the maid role took the plan and policy of the diva (2026-10-16).</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>curve P05</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 42% against Euthys on the engine corrected by the audit of 2026-10-18/19 (spells that miss deal half, the starting gauges and the AI as the program has them, the enchantments of the enemies counted): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 40, the stand-in of the model for that preparation, it wins 100% (dtcli crown-trial, 200 battles, 2026-10-19).</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>curve P25</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 68% against Mil the Overlord on the engine corrected by the audit of 2026-10-18/19 (spells that miss deal half, the starting gauges and the AI as the program has them, the enchantments of the enemies counted): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 40, the stand-in of the model for that preparation, it wins 100% (dtcli crown-trial, 200 battles, 2026-10-19).</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>curve P28</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 38% against Hell's Angel on the engine corrected by the audit of 2026-10-18/19 (spells that miss deal half, the starting gauges and the AI as the program has them, the enchantments of the enemies counted): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 40, the stand-in of the model for that preparation, it wins 100% (dtcli crown-trial, 200 battles, 2026-10-19).</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>curve P31</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 2% against the weakened Matrix superboss on the engine corrected by the audit of 2026-10-18/19 (spells that miss deal half, the starting gauges and the AI as the program has them, the enchantments of the enemies counted): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 40, the stand-in of the model for that preparation, it wins 87% (dtcli crown-trial, 200 battles, 2026-10-19).</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>curve P44</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 8% against Yoshitsune of the Wandering Brigade on the engine corrected by the audit of 2026-10-18/19 (spells that miss deal half, the starting gauges and the AI as the program has them, the enchantments of the enemies counted): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 40, the stand-in of the model for that preparation, it wins 100% (dtcli crown-trial, 200 battles, 2026-10-19).</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>curve P52</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 8% against Bearerophon on the engine corrected by the audit of 2026-10-18/19 (spells that miss deal half, the starting gauges and the AI as the program has them, the enchantments of the enemies counted): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 40, the stand-in of the model for that preparation, it wins 98% (dtcli crown-trial, 200 battles, 2026-10-19).</t>
         </is>
       </c>
     </row>
@@ -19478,7 +19580,6 @@
           <t>boss_fit_skip</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
           <t>Checkpoints tools/boss_fit.py gentle leaves alone: none since 2026-10-19 (C29 is played with the guide's preparation, sheet CheckpointGuests)</t>

</xml_diff>

<commit_message>
sim: Soul Summoner role revives and casts Divine Shield
The role had no row to revive a fallen member with items and never cast
Divine Shield (skill 201, inherited from the Priestess line), though every
other support role does both. Class-search showed her parties with the
lowest of the lowest HP from C27 on. Two rows of the sheet Policies; the
golden traces are unchanged.
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -19682,7 +19682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E93"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -22016,6 +22016,56 @@
       <c r="E93" t="inlineStr">
         <is>
           <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>ally_down</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>revive</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>items when a member falls, as the other roles of the support line do (2026-10-19: the role had no row for it)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>boss</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>status:187</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>the class kit: Divine Shield (skill 201) of the Priestess line, prebuffed in hard fights as the other support roles prebuff their guards (2026-10-19: the role never cast it; class-search showed her parties the lowest of the lowest HP from C27 on)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sim: no buff kept up against foes that strip buffs
New policy condition no_foe_dispels: true while no living foe has an
attack with effect 74. The Kunoichi keeps Shadow Clone up only then: at
C33 (Death Cataphract, whose plain blow strips buffs) she spent the fight
casting it again and dealt almost no damage (a 50% stronger Ninja
Piledriver left 76 of 83 of her parties unchanged). Golden traces
unchanged.
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -20530,7 +20530,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>no_foe_dispels</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -20540,7 +20540,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Shadow Clone kept up (page 142)</t>
+          <t>Shadow Clone kept up (page 142) | 2026-10-19: not against foes whose attacks strip buffs (Death Cataphract, C33): she spent the fight casting it again after every plain blow and dealt almost no damage (class-search: a 50% stronger Ninja Piledriver left 76 of 83 Kunoichi parties of C33 unchanged)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(sim): Soul Summoner measured with Soul Seal (skill priority + realistic personal sealbooks C02-P05, tested role carries its sealbook)
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -16889,7 +16889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17147,7 +17147,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>soul summoner</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -17172,57 +17172,57 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>dolls</t>
+          <t>diva</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Persephone</t>
+          <t>Demi Lich</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>P06</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Demi Lich (level 69), "a pretty early sealbook", for the Diva and offensive mages</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>healer</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Persephone</t>
+          <t>Demi Lich</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>P06</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Demi Lich (level 69), "a pretty early sealbook", for the Diva and offensive mages</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>diva</t>
+          <t>mage</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -17247,7 +17247,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>healer</t>
+          <t>sage</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -17272,7 +17272,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>mage</t>
+          <t>magical princess</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -17297,7 +17297,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>sage</t>
+          <t>maid</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -17322,75 +17322,875 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>magical princess</t>
+          <t>etoile</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>453</v>
+        <v>56</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Demi Lich</t>
+          <t>Himiko</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Demi Lich (level 69), "a pretty early sealbook", for the Diva and offensive mages</t>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Himiko (level 81, a regular monster), top tier for the Etoile</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>maid</t>
+          <t>soul summoner</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>453</v>
+        <v>90</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Demi Lich</t>
+          <t>Ainsel</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>C02</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Demi Lich (level 69), "a pretty early sealbook", for the Diva and offensive mages</t>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>etoile</t>
+          <t>dolls</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>56</v>
+        <v>90</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Himiko</t>
+          <t>Ainsel</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>C02</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Himiko (level 81, a regular monster), top tier for the Etoile</t>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>84</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Spider Girl</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>C03</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>84</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Spider Girl</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>C03</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>823</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Bigtooth</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>C07</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>823</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Bigtooth</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>C07</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>342</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Creature</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>C08</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>342</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Creature</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>C08</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>743</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Selene</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>C09</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>743</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Selene</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>C09</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>193</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Eel</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>193</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Eel</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>772</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Korpokkur</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>C14</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>772</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Korpokkur</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>C14</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>141</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Demon</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>141</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Demon</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>433</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Skull Collector</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>C18</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>433</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Skull Collector</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>C18</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>715</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Psycher</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>715</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Psycher</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>845</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Ape</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>C24</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>845</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Ape</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>C24</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>393</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Dragonkin</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>C25</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>393</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Dragonkin</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>C25</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>101</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Kraken</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>C27</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>101</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Kraken</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>C27</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>182</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Momunofu</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>C28</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>182</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Momunofu</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>C28</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>891</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Gargouille</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>C29</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>891</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Gargouille</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>C29</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>910</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>910</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Derived: the strongest regular enemy (stat sum) of the floors reached before the checkpoint; a sealbook a player carries for Soul Seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>458</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Persephone</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>458</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Persephone</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
         </is>
       </c>
     </row>
@@ -23007,7 +23807,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Spartan; Catalina; Doll Mastery; Double Puppet; Mercidarian; Perdurabo; Musiy; Soul Eater; Oracles; Destiny Line; Coffee Break; Weapon Mastery; Danger Shoot</t>
+          <t>Spartan; Catalina; Doll Mastery; Double Puppet; Soul Seal; Mercidarian; Perdurabo; Musiy; Soul Eater; Oracles; Destiny Line; Coffee Break; Weapon Mastery; Danger Shoot</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">

</xml_diff>

<commit_message>
sim: rules for Catalina (dolls) and Armor Penetration (attacker)
Catalina is summoned when the party is below 60% HP; Armor Penetration is cast once in the first three turns. Trials at 16 bosses, 1000 battles each: Catalina wins +1.2 and no boss worse (every-turn rule: fights 16% longer); Armor Penetration 4 bosses served, 1 hurt (every-turn rule: 5 hurt). The skill battery moves it from dead to niche.
</commit_message>
<xml_diff>
--- a/data_tables/sim_setup.xlsx
+++ b/data_tables/sim_setup.xlsx
@@ -20482,7 +20482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -22866,6 +22866,56 @@
       <c r="E95" t="inlineStr">
         <is>
           <t>the class kit: Divine Shield (skill 201) of the Priestess line, prebuffed in hard fights as the other support roles prebuff their guards (2026-10-19: the role never cast it; class-search showed her parties the lowest of the lowest HP from C27 on)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>party_hp_below:0.6</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>skill:Catalina</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>skill-rule-trial of 2026-10-29 (16 bosses, 1000 battles each): Catalina summoned every time TP allowed cost the party 9 casts of 48 TP a battle (fights 16% longer, 6 of 16 bosses worse); summoned when the party is below 60% HP: wins +1.2 points, fights 0.9% longer, 0 bosses worse, 3 better by 3 points or more</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>turn_at_most:3</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>skill:Armor Penetration</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>skill-rule-trial of 2026-10-29 (16 bosses, 1000 battles each): the policy never chose it (38 - 44% of the damage per time of Moonlight Purgatory) but its DEF -24% to -38% for 4 turns serves the whole party; cast once at the start of a fight: wins +0.3 points, fights 1.5% shorter, 4 bosses served and 1 hurt, against 5 hurt when it is used every time</t>
         </is>
       </c>
     </row>

</xml_diff>